<commit_message>
Forms sync auto batch 5: 5000 files
</commit_message>
<xml_diff>
--- a/inspection_forms/020_logistics_audit_checklist--inspection_forms.xlsx
+++ b/inspection_forms/020_logistics_audit_checklist--inspection_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1198,8 +1198,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_'good'}</t>
+          <t>good</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': 'Good'}</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_'fair'}</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': 'Fair'}</t>
+          <t>Fair</t>
         </is>
       </c>
     </row>
@@ -1261,12 +1261,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{'id':_3,_'text':_'poor'}</t>
+          <t>poor</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'id': 3, 'text': 'Poor'}</t>
+          <t>Poor</t>
         </is>
       </c>
     </row>
@@ -1278,12 +1278,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_'on_time'}</t>
+          <t>on_time</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': 'On Time'}</t>
+          <t>On Time</t>
         </is>
       </c>
     </row>
@@ -1329,12 +1329,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_'behind_schedule'}</t>
+          <t>behind_schedule</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': 'Behind Schedule'}</t>
+          <t>Behind Schedule</t>
         </is>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1363,12 +1363,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1380,12 +1380,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1397,12 +1397,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1431,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1448,12 +1448,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1465,12 +1465,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1482,12 +1482,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1533,12 +1533,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1567,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1584,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1601,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1618,12 +1618,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1635,12 +1635,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1652,12 +1652,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1669,12 +1669,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1703,12 +1703,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1771,12 +1771,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1890,12 +1890,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1907,12 +1907,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1924,12 +1924,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1941,12 +1941,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1958,12 +1958,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -1992,12 +1992,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_true}</t>
+          <t>true</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': True}</t>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_false}</t>
+          <t>false</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': False}</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -2026,12 +2026,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>{'id':_1,_'text':_'daily'}</t>
+          <t>daily</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>{'id': 1, 'text': 'Daily'}</t>
+          <t>Daily</t>
         </is>
       </c>
     </row>
@@ -2043,12 +2043,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>{'id':_2,_'text':_'weekly'}</t>
+          <t>weekly</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>{'id': 2, 'text': 'Weekly'}</t>
+          <t>Weekly</t>
         </is>
       </c>
     </row>
@@ -2060,12 +2060,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>{'id':_3,_'text':_'monthly'}</t>
+          <t>monthly</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>{'id': 3, 'text': 'Monthly'}</t>
+          <t>Monthly</t>
         </is>
       </c>
     </row>
@@ -2077,12 +2077,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>{'id':_4,_'text':_'quarterly'}</t>
+          <t>quarterly</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>{'id': 4, 'text': 'Quarterly'}</t>
+          <t>Quarterly</t>
         </is>
       </c>
     </row>
@@ -2094,12 +2094,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{'id':_5,_'text':_'semi-annually'}</t>
+          <t>semi-annually</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>{'id': 5, 'text': 'Semi-Annually'}</t>
+          <t>Semi-Annually</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>{'id':_6,_'text':_'annually'}</t>
+          <t>annually</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>{'id': 6, 'text': 'Annually'}</t>
+          <t>Annually</t>
         </is>
       </c>
     </row>

</xml_diff>